<commit_message>
Refactor r_inad function to consolidate paths for inadimplência files; enhance data extraction for recent entries; update documentation for clarity.
</commit_message>
<xml_diff>
--- a/dados/Contas x CNPJs - VItor.xlsx
+++ b/dados/Contas x CNPJs - VItor.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla-my.sharepoint.com/personal/vitor_amplaincorporadora_com_br/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla.sharepoint.com/sites/Controladoria/Documentos Compartilhados/amplaGitHub/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{06233A17-DE62-45C5-A675-F79EDA089E2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DD674C2-05C4-42AF-9464-6A3266DBB384}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{06233A17-DE62-45C5-A675-F79EDA089E2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B0F92F5-85FE-4CB7-A526-8ABDCC96D18D}"/>
   <bookViews>
-    <workbookView xWindow="-43200" yWindow="-3555" windowWidth="14400" windowHeight="15600" xr2:uid="{17DF5601-8A24-4FB8-9E43-44A7D47D4957}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{17DF5601-8A24-4FB8-9E43-44A7D47D4957}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -2585,6 +2585,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36569ac63cfce8ff0f8884bc80e67f1c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2040da04b75a9ea4fe796fa8180f8ca6" ns2:_="" ns3:_="">
     <xsd:import namespace="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
@@ -2779,15 +2788,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2800,13 +2800,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A6FDE2E-1858-4113-9CEB-EA62B374FDA2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45FBC689-CC2B-4454-9877-FD3585F7B392}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45FBC689-CC2B-4454-9877-FD3585F7B392}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A6FDE2E-1858-4113-9CEB-EA62B374FDA2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
+    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D0116357-0756-4F4A-86B8-48D9AFAC169A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D0116357-0756-4F4A-86B8-48D9AFAC169A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
+    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>